<commit_message>
Pont build_metre vers gabarit 5 feuilles + injecteur dynamique
- build_metre.py : MetreGenerator(plan_data, moteur=gabarit/historique),
  adaptateur plan_data->plat, chemin template frozen-aware, CLI --dxf/--json/--moteur
- core/populate_modele.py : allocation dynamique (N semelles, poteaux,
  poutres), sous-totaux et liens feuille 4 recalcules, bloc futs
- core/local_extractor.py : dedupe groupes identiques (_dedupe_bars),
  4T12+4T10 conserves, 629.7 kg valides
- build_executable.py : gabarit embarque (templates/, regenere si absent)
- tests/test_pont_gabarit.py : 11 tests pont (adaptateur, frozen,
  regeneration, dynamique, liens)
- tests/test_build_metre.py : moteur historique explicite
- outputs regeneres (metre 5 feuilles, template catalogue, plan_data)
</commit_message>
<xml_diff>
--- a/output/modele_metre_BA.xlsx
+++ b/output/modele_metre_BA.xlsx
@@ -11,6 +11,7 @@
     <sheet name="02_Armatures" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="03_Attachement_Ferraillage" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="04_GO_Attachement" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="05_Catalogue_Armatures_Standard" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,11 +20,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="#,##0.000"/>
-    <numFmt numFmtId="165" formatCode="0.0%"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -71,8 +71,20 @@
       <color rgb="000F172A"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <i val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001B365D"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -109,8 +121,14 @@
         <bgColor rgb="000D9488"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2E8F0"/>
+        <bgColor rgb="00E2E8F0"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -146,11 +164,55 @@
         <color rgb="001B365D"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D1D5DB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D1D5DB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D1D5DB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D1D5DB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D1D5DB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D1D5DB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D1D5DB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D1D5DB"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -213,8 +275,38 @@
     <xf numFmtId="4" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -610,18 +702,23 @@
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
+      <c r="C2" s="34" t="n"/>
       <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Projet :</t>
         </is>
       </c>
       <c r="E2" s="3" t="n"/>
+      <c r="F2" s="35" t="n"/>
+      <c r="G2" s="34" t="n"/>
       <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Bâtiment :</t>
         </is>
       </c>
       <c r="I2" s="3" t="n"/>
+      <c r="J2" s="35" t="n"/>
+      <c r="K2" s="34" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -630,18 +727,23 @@
         </is>
       </c>
       <c r="B3" s="3" t="n"/>
+      <c r="C3" s="34" t="n"/>
       <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Établi par :</t>
         </is>
       </c>
       <c r="E3" s="3" t="n"/>
+      <c r="F3" s="35" t="n"/>
+      <c r="G3" s="34" t="n"/>
       <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Vérifié par :</t>
         </is>
       </c>
       <c r="I3" s="3" t="n"/>
+      <c r="J3" s="35" t="n"/>
+      <c r="K3" s="34" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
@@ -1362,18 +1464,27 @@
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
+      <c r="C2" s="35" t="n"/>
+      <c r="D2" s="35" t="n"/>
+      <c r="E2" s="35" t="n"/>
+      <c r="F2" s="34" t="n"/>
       <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Date :</t>
         </is>
       </c>
       <c r="L2" s="3" t="n"/>
+      <c r="M2" s="35" t="n"/>
+      <c r="N2" s="34" t="n"/>
       <c r="O2" s="2" t="inlineStr">
         <is>
           <t>Indice :</t>
         </is>
       </c>
       <c r="P2" s="3" t="n"/>
+      <c r="Q2" s="35" t="n"/>
+      <c r="R2" s="35" t="n"/>
+      <c r="S2" s="34" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -2497,18 +2608,27 @@
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
+      <c r="C2" s="35" t="n"/>
+      <c r="D2" s="35" t="n"/>
+      <c r="E2" s="34" t="n"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Attachement n° :</t>
         </is>
       </c>
       <c r="G2" s="3" t="n"/>
+      <c r="H2" s="35" t="n"/>
+      <c r="I2" s="34" t="n"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
           <t>Date :</t>
         </is>
       </c>
       <c r="K2" s="3" t="n"/>
+      <c r="L2" s="35" t="n"/>
+      <c r="M2" s="35" t="n"/>
+      <c r="N2" s="35" t="n"/>
+      <c r="O2" s="34" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -3229,6 +3349,7 @@
         </is>
       </c>
       <c r="F2" s="3" t="n"/>
+      <c r="G2" s="34" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -3292,7 +3413,7 @@
         <f>D4-E4</f>
         <v/>
       </c>
-      <c r="G4" s="32">
+      <c r="G4" s="36">
         <f>IF(D4&gt;0,E4/D4,0)</f>
         <v/>
       </c>
@@ -3322,7 +3443,7 @@
         <f>D5-E5</f>
         <v/>
       </c>
-      <c r="G5" s="32">
+      <c r="G5" s="36">
         <f>IF(D5&gt;0,E5/D5,0)</f>
         <v/>
       </c>
@@ -3352,7 +3473,7 @@
         <f>D6-E6</f>
         <v/>
       </c>
-      <c r="G6" s="32">
+      <c r="G6" s="36">
         <f>IF(D6&gt;0,E6/D6,0)</f>
         <v/>
       </c>
@@ -3382,7 +3503,7 @@
         <f>D7-E7</f>
         <v/>
       </c>
-      <c r="G7" s="32">
+      <c r="G7" s="36">
         <f>IF(D7&gt;0,E7/D7,0)</f>
         <v/>
       </c>
@@ -3396,4 +3517,2635 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K64"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="37" t="inlineStr">
+        <is>
+          <t>RÉFÉRENTIEL TECHNIQUE — CATALOGUE DES ARMATURES STANDARDISÉES (FIMUREX / EUROCODE 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="38" t="inlineStr">
+        <is>
+          <t>Abaques de dimensionnement, sections d'acier, charges admissibles et nomenclatures de chantier</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="39" t="inlineStr">
+        <is>
+          <t>1. POTEAUX PRÉFABRIQUÉS STANDARD (FIMUREX PN - 4 ET 6 FILANTS, H &lt;= 2.80 m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="40" t="inlineStr">
+        <is>
+          <t>Réf. Armature</t>
+        </is>
+      </c>
+      <c r="B5" s="40" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C5" s="40" t="inlineStr">
+        <is>
+          <t>Section Béton (cm)</t>
+        </is>
+      </c>
+      <c r="D5" s="40" t="inlineStr">
+        <is>
+          <t>Aciers Filants</t>
+        </is>
+      </c>
+      <c r="E5" s="40" t="inlineStr">
+        <is>
+          <t>Cadres / Espac.</t>
+        </is>
+      </c>
+      <c r="F5" s="40" t="inlineStr">
+        <is>
+          <t>Pser Intérieur (daN)</t>
+        </is>
+      </c>
+      <c r="G5" s="40" t="inlineStr">
+        <is>
+          <t>Pser Extérieur (daN)</t>
+        </is>
+      </c>
+      <c r="H5" s="40" t="inlineStr">
+        <is>
+          <t>Pser Int. (kN)</t>
+        </is>
+      </c>
+      <c r="I5" s="40" t="inlineStr">
+        <is>
+          <t>Pser Ext. (kN)</t>
+        </is>
+      </c>
+      <c r="J5" s="40" t="inlineStr">
+        <is>
+          <t>Attente PA</t>
+        </is>
+      </c>
+      <c r="K5" s="40" t="inlineStr">
+        <is>
+          <t>Domaine / Norme</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="41" t="inlineStr">
+        <is>
+          <t>PN4108X8</t>
+        </is>
+      </c>
+      <c r="B6" s="41" t="inlineStr">
+        <is>
+          <t>Type I</t>
+        </is>
+      </c>
+      <c r="C6" s="41" t="inlineStr">
+        <is>
+          <t>15 x 15</t>
+        </is>
+      </c>
+      <c r="D6" s="41" t="inlineStr">
+        <is>
+          <t>4 HA 10</t>
+        </is>
+      </c>
+      <c r="E6" s="41" t="inlineStr">
+        <is>
+          <t>HA 5 e=15</t>
+        </is>
+      </c>
+      <c r="F6" s="42" t="n">
+        <v>11780</v>
+      </c>
+      <c r="G6" s="42" t="n">
+        <v>19500</v>
+      </c>
+      <c r="H6" s="42" t="n">
+        <v>117.8</v>
+      </c>
+      <c r="I6" s="42" t="n">
+        <v>195</v>
+      </c>
+      <c r="J6" s="41" t="inlineStr">
+        <is>
+          <t>PA4108X8</t>
+        </is>
+      </c>
+      <c r="K6" s="43" t="inlineStr">
+        <is>
+          <t>Eurocode 2 / Non sismique</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="41" t="inlineStr">
+        <is>
+          <t>PN41010X10</t>
+        </is>
+      </c>
+      <c r="B7" s="41" t="inlineStr">
+        <is>
+          <t>Type I</t>
+        </is>
+      </c>
+      <c r="C7" s="41" t="inlineStr">
+        <is>
+          <t>15 x 15</t>
+        </is>
+      </c>
+      <c r="D7" s="41" t="inlineStr">
+        <is>
+          <t>4 HA 10</t>
+        </is>
+      </c>
+      <c r="E7" s="41" t="inlineStr">
+        <is>
+          <t>HA 5 e=15</t>
+        </is>
+      </c>
+      <c r="F7" s="42" t="n">
+        <v>11840</v>
+      </c>
+      <c r="G7" s="42" t="n">
+        <v>25650</v>
+      </c>
+      <c r="H7" s="42" t="n">
+        <v>118.4</v>
+      </c>
+      <c r="I7" s="42" t="n">
+        <v>256.5</v>
+      </c>
+      <c r="J7" s="41" t="inlineStr">
+        <is>
+          <t>PA41010X10</t>
+        </is>
+      </c>
+      <c r="K7" s="43" t="inlineStr">
+        <is>
+          <t>Eurocode 2 / Non sismique</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="41" t="inlineStr">
+        <is>
+          <t>PN41015X15</t>
+        </is>
+      </c>
+      <c r="B8" s="41" t="inlineStr">
+        <is>
+          <t>Type I</t>
+        </is>
+      </c>
+      <c r="C8" s="41" t="inlineStr">
+        <is>
+          <t>20 x 20</t>
+        </is>
+      </c>
+      <c r="D8" s="41" t="inlineStr">
+        <is>
+          <t>4 HA 10</t>
+        </is>
+      </c>
+      <c r="E8" s="41" t="inlineStr">
+        <is>
+          <t>HA 5 e=15</t>
+        </is>
+      </c>
+      <c r="F8" s="42" t="n">
+        <v>25810</v>
+      </c>
+      <c r="G8" s="42" t="n">
+        <v>45180</v>
+      </c>
+      <c r="H8" s="42" t="n">
+        <v>258.1</v>
+      </c>
+      <c r="I8" s="42" t="n">
+        <v>451.8</v>
+      </c>
+      <c r="J8" s="41" t="inlineStr">
+        <is>
+          <t>PA1015X15</t>
+        </is>
+      </c>
+      <c r="K8" s="43" t="inlineStr">
+        <is>
+          <t>Eurocode 2 / Non sismique</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="41" t="inlineStr">
+        <is>
+          <t>PN41020X20</t>
+        </is>
+      </c>
+      <c r="B9" s="41" t="inlineStr">
+        <is>
+          <t>Type I</t>
+        </is>
+      </c>
+      <c r="C9" s="41" t="inlineStr">
+        <is>
+          <t>25 x 25</t>
+        </is>
+      </c>
+      <c r="D9" s="41" t="inlineStr">
+        <is>
+          <t>4 HA 10</t>
+        </is>
+      </c>
+      <c r="E9" s="41" t="inlineStr">
+        <is>
+          <t>HA 5 e=15</t>
+        </is>
+      </c>
+      <c r="F9" s="42" t="n">
+        <v>45320</v>
+      </c>
+      <c r="G9" s="42" t="n">
+        <v>70840</v>
+      </c>
+      <c r="H9" s="42" t="n">
+        <v>453.2</v>
+      </c>
+      <c r="I9" s="42" t="n">
+        <v>708.4</v>
+      </c>
+      <c r="J9" s="41" t="inlineStr">
+        <is>
+          <t>PA1015X15</t>
+        </is>
+      </c>
+      <c r="K9" s="43" t="inlineStr">
+        <is>
+          <t>Eurocode 2 / Non sismique</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="41" t="inlineStr">
+        <is>
+          <t>P6N41025X25</t>
+        </is>
+      </c>
+      <c r="B10" s="41" t="inlineStr">
+        <is>
+          <t>Type I</t>
+        </is>
+      </c>
+      <c r="C10" s="41" t="inlineStr">
+        <is>
+          <t>30 x 30</t>
+        </is>
+      </c>
+      <c r="D10" s="41" t="inlineStr">
+        <is>
+          <t>4 HA 10</t>
+        </is>
+      </c>
+      <c r="E10" s="41" t="inlineStr">
+        <is>
+          <t>HA 5 e=15</t>
+        </is>
+      </c>
+      <c r="F10" s="42" t="n">
+        <v>70960</v>
+      </c>
+      <c r="G10" s="42" t="n">
+        <v>97560</v>
+      </c>
+      <c r="H10" s="42" t="n">
+        <v>709.6</v>
+      </c>
+      <c r="I10" s="42" t="n">
+        <v>975.6</v>
+      </c>
+      <c r="J10" s="41" t="inlineStr">
+        <is>
+          <t>Sur mesure</t>
+        </is>
+      </c>
+      <c r="K10" s="43" t="inlineStr">
+        <is>
+          <t>Eurocode 2 / Non sismique</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="41" t="inlineStr">
+        <is>
+          <t>PN41010X20</t>
+        </is>
+      </c>
+      <c r="B11" s="41" t="inlineStr">
+        <is>
+          <t>Type I</t>
+        </is>
+      </c>
+      <c r="C11" s="41" t="inlineStr">
+        <is>
+          <t>15 x 25</t>
+        </is>
+      </c>
+      <c r="D11" s="41" t="inlineStr">
+        <is>
+          <t>4 HA 10</t>
+        </is>
+      </c>
+      <c r="E11" s="41" t="inlineStr">
+        <is>
+          <t>HA 5 e=15</t>
+        </is>
+      </c>
+      <c r="F11" s="42" t="n">
+        <v>17770</v>
+      </c>
+      <c r="G11" s="42" t="n">
+        <v>36470</v>
+      </c>
+      <c r="H11" s="42" t="n">
+        <v>177.7</v>
+      </c>
+      <c r="I11" s="42" t="n">
+        <v>364.7</v>
+      </c>
+      <c r="J11" s="41" t="inlineStr">
+        <is>
+          <t>PA41010X10</t>
+        </is>
+      </c>
+      <c r="K11" s="43" t="inlineStr">
+        <is>
+          <t>Eurocode 2 / Section rect.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="41" t="inlineStr">
+        <is>
+          <t>PN41015X20</t>
+        </is>
+      </c>
+      <c r="B12" s="41" t="inlineStr">
+        <is>
+          <t>Type I</t>
+        </is>
+      </c>
+      <c r="C12" s="41" t="inlineStr">
+        <is>
+          <t>20 x 25</t>
+        </is>
+      </c>
+      <c r="D12" s="41" t="inlineStr">
+        <is>
+          <t>4 HA 10</t>
+        </is>
+      </c>
+      <c r="E12" s="41" t="inlineStr">
+        <is>
+          <t>HA 5 e=15</t>
+        </is>
+      </c>
+      <c r="F12" s="42" t="n">
+        <v>31210</v>
+      </c>
+      <c r="G12" s="42" t="n">
+        <v>53230</v>
+      </c>
+      <c r="H12" s="42" t="n">
+        <v>312.1</v>
+      </c>
+      <c r="I12" s="42" t="n">
+        <v>532.3</v>
+      </c>
+      <c r="J12" s="41" t="inlineStr">
+        <is>
+          <t>PA1015X15</t>
+        </is>
+      </c>
+      <c r="K12" s="43" t="inlineStr">
+        <is>
+          <t>Eurocode 2 / Section rect.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="41" t="inlineStr">
+        <is>
+          <t>P6N61015X30</t>
+        </is>
+      </c>
+      <c r="B13" s="41" t="inlineStr">
+        <is>
+          <t>Type III</t>
+        </is>
+      </c>
+      <c r="C13" s="41" t="inlineStr">
+        <is>
+          <t>20 x 35</t>
+        </is>
+      </c>
+      <c r="D13" s="41" t="inlineStr">
+        <is>
+          <t>6 HA 10</t>
+        </is>
+      </c>
+      <c r="E13" s="41" t="inlineStr">
+        <is>
+          <t>HA 5 e=15</t>
+        </is>
+      </c>
+      <c r="F13" s="42" t="n">
+        <v>42010</v>
+      </c>
+      <c r="G13" s="42" t="n">
+        <v>69330</v>
+      </c>
+      <c r="H13" s="42" t="n">
+        <v>420.1</v>
+      </c>
+      <c r="I13" s="42" t="n">
+        <v>693.3</v>
+      </c>
+      <c r="J13" s="41" t="inlineStr">
+        <is>
+          <t>PA661010X25</t>
+        </is>
+      </c>
+      <c r="K13" s="43" t="inlineStr">
+        <is>
+          <t>Eurocode 2 / 6 filants</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="41" t="inlineStr">
+        <is>
+          <t>P6N61015X40</t>
+        </is>
+      </c>
+      <c r="B14" s="41" t="inlineStr">
+        <is>
+          <t>Type III</t>
+        </is>
+      </c>
+      <c r="C14" s="41" t="inlineStr">
+        <is>
+          <t>20 x 45</t>
+        </is>
+      </c>
+      <c r="D14" s="41" t="inlineStr">
+        <is>
+          <t>6 HA 10</t>
+        </is>
+      </c>
+      <c r="E14" s="41" t="inlineStr">
+        <is>
+          <t>HA 5 e=15</t>
+        </is>
+      </c>
+      <c r="F14" s="42" t="n">
+        <v>52820</v>
+      </c>
+      <c r="G14" s="42" t="n">
+        <v>85430</v>
+      </c>
+      <c r="H14" s="42" t="n">
+        <v>528.2</v>
+      </c>
+      <c r="I14" s="42" t="n">
+        <v>854.3</v>
+      </c>
+      <c r="J14" s="41" t="inlineStr">
+        <is>
+          <t>PA661010X35</t>
+        </is>
+      </c>
+      <c r="K14" s="43" t="inlineStr">
+        <is>
+          <t>Eurocode 2 / 6 filants</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="39" t="inlineStr">
+        <is>
+          <t>2. SEMELLES ISOLÉES SOUS POTEAUX (FIMUREX SIC CARRÉES)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="40" t="inlineStr">
+        <is>
+          <t>Réf. Armature</t>
+        </is>
+      </c>
+      <c r="B17" s="40" t="inlineStr">
+        <is>
+          <t>Section AxAxH (cm)</t>
+        </is>
+      </c>
+      <c r="C17" s="40" t="inlineStr">
+        <is>
+          <t>Pser à 1.0 bar (daN)</t>
+        </is>
+      </c>
+      <c r="D17" s="40" t="inlineStr">
+        <is>
+          <t>Pser à 1.5 bar (daN)</t>
+        </is>
+      </c>
+      <c r="E17" s="40" t="inlineStr">
+        <is>
+          <t>Pser à 2.0 bars (daN)</t>
+        </is>
+      </c>
+      <c r="F17" s="40" t="inlineStr">
+        <is>
+          <t>Pser 1.5b (kN)</t>
+        </is>
+      </c>
+      <c r="G17" s="40" t="inlineStr">
+        <is>
+          <t>Nappes Inf. X</t>
+        </is>
+      </c>
+      <c r="H17" s="40" t="inlineStr">
+        <is>
+          <t>Nappes Inf. Y</t>
+        </is>
+      </c>
+      <c r="I17" s="40" t="inlineStr">
+        <is>
+          <t>Crochets (e cm)</t>
+        </is>
+      </c>
+      <c r="J17" s="40" t="inlineStr">
+        <is>
+          <t>Abouts (cm)</t>
+        </is>
+      </c>
+      <c r="K17" s="40" t="inlineStr">
+        <is>
+          <t>Enrobage (cm)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="41" t="inlineStr">
+        <is>
+          <t>SIC4655 / 4855</t>
+        </is>
+      </c>
+      <c r="B18" s="41" t="inlineStr">
+        <is>
+          <t>65 x 65 x 20</t>
+        </is>
+      </c>
+      <c r="C18" s="42" t="n">
+        <v>4230</v>
+      </c>
+      <c r="D18" s="42" t="n">
+        <v>6340</v>
+      </c>
+      <c r="E18" s="42" t="n">
+        <v>8450</v>
+      </c>
+      <c r="F18" s="44" t="n">
+        <v>63.4</v>
+      </c>
+      <c r="G18" s="41" t="inlineStr">
+        <is>
+          <t>4 HA 8</t>
+        </is>
+      </c>
+      <c r="H18" s="41" t="inlineStr">
+        <is>
+          <t>4 HA 8</t>
+        </is>
+      </c>
+      <c r="I18" s="41" t="inlineStr">
+        <is>
+          <t>e = 15</t>
+        </is>
+      </c>
+      <c r="J18" s="45" t="n">
+        <v>5</v>
+      </c>
+      <c r="K18" s="45" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="41" t="inlineStr">
+        <is>
+          <t>SIC5775</t>
+        </is>
+      </c>
+      <c r="B19" s="41" t="inlineStr">
+        <is>
+          <t>85 x 85 x 25</t>
+        </is>
+      </c>
+      <c r="C19" s="42" t="n">
+        <v>7230</v>
+      </c>
+      <c r="D19" s="42" t="n">
+        <v>10840</v>
+      </c>
+      <c r="E19" s="42" t="n">
+        <v>14450</v>
+      </c>
+      <c r="F19" s="42" t="n">
+        <v>108.4</v>
+      </c>
+      <c r="G19" s="41" t="inlineStr">
+        <is>
+          <t>5 HA 8</t>
+        </is>
+      </c>
+      <c r="H19" s="41" t="inlineStr">
+        <is>
+          <t>5 HA 8</t>
+        </is>
+      </c>
+      <c r="I19" s="41" t="inlineStr">
+        <is>
+          <t>e = 15</t>
+        </is>
+      </c>
+      <c r="J19" s="45" t="n">
+        <v>5</v>
+      </c>
+      <c r="K19" s="45" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="41" t="inlineStr">
+        <is>
+          <t>SIC6895</t>
+        </is>
+      </c>
+      <c r="B20" s="41" t="inlineStr">
+        <is>
+          <t>105 x 105 x 30</t>
+        </is>
+      </c>
+      <c r="C20" s="42" t="n">
+        <v>11030</v>
+      </c>
+      <c r="D20" s="42" t="n">
+        <v>16540</v>
+      </c>
+      <c r="E20" s="42" t="n">
+        <v>22050</v>
+      </c>
+      <c r="F20" s="42" t="n">
+        <v>165.4</v>
+      </c>
+      <c r="G20" s="41" t="inlineStr">
+        <is>
+          <t>6 HA 8</t>
+        </is>
+      </c>
+      <c r="H20" s="41" t="inlineStr">
+        <is>
+          <t>6 HA 8</t>
+        </is>
+      </c>
+      <c r="I20" s="41" t="inlineStr">
+        <is>
+          <t>e = 15</t>
+        </is>
+      </c>
+      <c r="J20" s="45" t="n">
+        <v>5</v>
+      </c>
+      <c r="K20" s="45" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="41" t="inlineStr">
+        <is>
+          <t>SIC610115</t>
+        </is>
+      </c>
+      <c r="B21" s="41" t="inlineStr">
+        <is>
+          <t>125 x 125 x 35</t>
+        </is>
+      </c>
+      <c r="C21" s="42" t="n">
+        <v>15630</v>
+      </c>
+      <c r="D21" s="42" t="n">
+        <v>23440</v>
+      </c>
+      <c r="E21" s="42" t="n">
+        <v>31250</v>
+      </c>
+      <c r="F21" s="42" t="n">
+        <v>234.4</v>
+      </c>
+      <c r="G21" s="41" t="inlineStr">
+        <is>
+          <t>6 HA 10</t>
+        </is>
+      </c>
+      <c r="H21" s="41" t="inlineStr">
+        <is>
+          <t>6 HA 10</t>
+        </is>
+      </c>
+      <c r="I21" s="41" t="inlineStr">
+        <is>
+          <t>e = 15</t>
+        </is>
+      </c>
+      <c r="J21" s="45" t="n">
+        <v>5</v>
+      </c>
+      <c r="K21" s="45" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="41" t="inlineStr">
+        <is>
+          <t>SIC710135</t>
+        </is>
+      </c>
+      <c r="B22" s="41" t="inlineStr">
+        <is>
+          <t>145 x 145 x 40</t>
+        </is>
+      </c>
+      <c r="C22" s="42" t="n">
+        <v>21030</v>
+      </c>
+      <c r="D22" s="42" t="n">
+        <v>31540</v>
+      </c>
+      <c r="E22" s="42" t="n">
+        <v>38090</v>
+      </c>
+      <c r="F22" s="42" t="n">
+        <v>315.4</v>
+      </c>
+      <c r="G22" s="41" t="inlineStr">
+        <is>
+          <t>7 HA 10</t>
+        </is>
+      </c>
+      <c r="H22" s="41" t="inlineStr">
+        <is>
+          <t>7 HA 10</t>
+        </is>
+      </c>
+      <c r="I22" s="41" t="inlineStr">
+        <is>
+          <t>e = 15</t>
+        </is>
+      </c>
+      <c r="J22" s="45" t="n">
+        <v>5</v>
+      </c>
+      <c r="K22" s="45" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="39" t="inlineStr">
+        <is>
+          <t>3. SEMELLES FILANTES PLATES &amp; RENFORCÉES (FIMUREX S / F / FM - Lg = 6.00 m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="40" t="inlineStr">
+        <is>
+          <t>Réf. Armature</t>
+        </is>
+      </c>
+      <c r="B25" s="40" t="inlineStr">
+        <is>
+          <t>Type Ouvrage</t>
+        </is>
+      </c>
+      <c r="C25" s="40" t="inlineStr">
+        <is>
+          <t>Largeur (cm)</t>
+        </is>
+      </c>
+      <c r="D25" s="40" t="inlineStr">
+        <is>
+          <t>Hauteur (cm)</t>
+        </is>
+      </c>
+      <c r="E25" s="40" t="inlineStr">
+        <is>
+          <t>Aciers Filants</t>
+        </is>
+      </c>
+      <c r="F25" s="40" t="inlineStr">
+        <is>
+          <t>Armatures Transv.</t>
+        </is>
+      </c>
+      <c r="G25" s="40" t="inlineStr">
+        <is>
+          <t>Espac. (cm)</t>
+        </is>
+      </c>
+      <c r="H25" s="40" t="inlineStr">
+        <is>
+          <t>Nuance Acier</t>
+        </is>
+      </c>
+      <c r="I25" s="40" t="inlineStr">
+        <is>
+          <t>Conditionnement</t>
+        </is>
+      </c>
+      <c r="J25" s="40" t="inlineStr">
+        <is>
+          <t>Usage Sol Recommandé</t>
+        </is>
+      </c>
+      <c r="K25" s="40" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="41" t="inlineStr">
+        <is>
+          <t>S3835</t>
+        </is>
+      </c>
+      <c r="B26" s="41" t="inlineStr">
+        <is>
+          <t>Semelle plate</t>
+        </is>
+      </c>
+      <c r="C26" s="45" t="n">
+        <v>35</v>
+      </c>
+      <c r="D26" s="45" t="n">
+        <v>5</v>
+      </c>
+      <c r="E26" s="41" t="inlineStr">
+        <is>
+          <t>3 HA 8</t>
+        </is>
+      </c>
+      <c r="F26" s="41" t="inlineStr">
+        <is>
+          <t>Crochets HA 5</t>
+        </is>
+      </c>
+      <c r="G26" s="41" t="inlineStr">
+        <is>
+          <t>e = 30</t>
+        </is>
+      </c>
+      <c r="H26" s="41" t="inlineStr">
+        <is>
+          <t>B500A / B500B</t>
+        </is>
+      </c>
+      <c r="I26" s="41" t="inlineStr">
+        <is>
+          <t>48 unités</t>
+        </is>
+      </c>
+      <c r="J26" s="43" t="inlineStr">
+        <is>
+          <t>Sol homogène sans tassement</t>
+        </is>
+      </c>
+      <c r="K26" s="41" t="inlineStr">
+        <is>
+          <t>EC2 / FD P18-717</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="41" t="inlineStr">
+        <is>
+          <t>S31040</t>
+        </is>
+      </c>
+      <c r="B27" s="41" t="inlineStr">
+        <is>
+          <t>Semelle plate</t>
+        </is>
+      </c>
+      <c r="C27" s="45" t="n">
+        <v>40</v>
+      </c>
+      <c r="D27" s="45" t="n">
+        <v>5</v>
+      </c>
+      <c r="E27" s="41" t="inlineStr">
+        <is>
+          <t>3 HA 10</t>
+        </is>
+      </c>
+      <c r="F27" s="41" t="inlineStr">
+        <is>
+          <t>Crochets HA 5</t>
+        </is>
+      </c>
+      <c r="G27" s="41" t="inlineStr">
+        <is>
+          <t>e = 30</t>
+        </is>
+      </c>
+      <c r="H27" s="41" t="inlineStr">
+        <is>
+          <t>B500A / B500B</t>
+        </is>
+      </c>
+      <c r="I27" s="41" t="inlineStr">
+        <is>
+          <t>48 unités</t>
+        </is>
+      </c>
+      <c r="J27" s="43" t="inlineStr">
+        <is>
+          <t>Sol homogène standard</t>
+        </is>
+      </c>
+      <c r="K27" s="41" t="inlineStr">
+        <is>
+          <t>EC2 / FD P18-717</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="41" t="inlineStr">
+        <is>
+          <t>S41050</t>
+        </is>
+      </c>
+      <c r="B28" s="41" t="inlineStr">
+        <is>
+          <t>Semelle plate</t>
+        </is>
+      </c>
+      <c r="C28" s="45" t="n">
+        <v>50</v>
+      </c>
+      <c r="D28" s="45" t="n">
+        <v>5</v>
+      </c>
+      <c r="E28" s="41" t="inlineStr">
+        <is>
+          <t>4 HA 10</t>
+        </is>
+      </c>
+      <c r="F28" s="41" t="inlineStr">
+        <is>
+          <t>Crochets HA 5</t>
+        </is>
+      </c>
+      <c r="G28" s="41" t="inlineStr">
+        <is>
+          <t>e = 30</t>
+        </is>
+      </c>
+      <c r="H28" s="41" t="inlineStr">
+        <is>
+          <t>B500A / B500B</t>
+        </is>
+      </c>
+      <c r="I28" s="41" t="inlineStr">
+        <is>
+          <t>48 unités</t>
+        </is>
+      </c>
+      <c r="J28" s="43" t="inlineStr">
+        <is>
+          <t>Murs porteurs lourds</t>
+        </is>
+      </c>
+      <c r="K28" s="41" t="inlineStr">
+        <is>
+          <t>EC2 / FD P18-717</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="41" t="inlineStr">
+        <is>
+          <t>F6835X15</t>
+        </is>
+      </c>
+      <c r="B29" s="41" t="inlineStr">
+        <is>
+          <t>Semelle renforcée</t>
+        </is>
+      </c>
+      <c r="C29" s="45" t="n">
+        <v>35</v>
+      </c>
+      <c r="D29" s="45" t="n">
+        <v>15</v>
+      </c>
+      <c r="E29" s="41" t="inlineStr">
+        <is>
+          <t>6 HA 8 (2 nappes)</t>
+        </is>
+      </c>
+      <c r="F29" s="41" t="inlineStr">
+        <is>
+          <t>Cadres HA 5</t>
+        </is>
+      </c>
+      <c r="G29" s="41" t="inlineStr">
+        <is>
+          <t>e = 30</t>
+        </is>
+      </c>
+      <c r="H29" s="41" t="inlineStr">
+        <is>
+          <t>B500B</t>
+        </is>
+      </c>
+      <c r="I29" s="41" t="inlineStr">
+        <is>
+          <t>8 unités</t>
+        </is>
+      </c>
+      <c r="J29" s="43" t="inlineStr">
+        <is>
+          <t>Faibles tassements diff.</t>
+        </is>
+      </c>
+      <c r="K29" s="41" t="inlineStr">
+        <is>
+          <t>EC2 / FD P18-717</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="41" t="inlineStr">
+        <is>
+          <t>F6835X20</t>
+        </is>
+      </c>
+      <c r="B30" s="41" t="inlineStr">
+        <is>
+          <t>Semelle renforcée</t>
+        </is>
+      </c>
+      <c r="C30" s="45" t="n">
+        <v>35</v>
+      </c>
+      <c r="D30" s="45" t="n">
+        <v>20</v>
+      </c>
+      <c r="E30" s="41" t="inlineStr">
+        <is>
+          <t>6 HA 8 (2 nappes)</t>
+        </is>
+      </c>
+      <c r="F30" s="41" t="inlineStr">
+        <is>
+          <t>Cadres HA 5</t>
+        </is>
+      </c>
+      <c r="G30" s="41" t="inlineStr">
+        <is>
+          <t>e = 30</t>
+        </is>
+      </c>
+      <c r="H30" s="41" t="inlineStr">
+        <is>
+          <t>B500B</t>
+        </is>
+      </c>
+      <c r="I30" s="41" t="inlineStr">
+        <is>
+          <t>6 unités</t>
+        </is>
+      </c>
+      <c r="J30" s="43" t="inlineStr">
+        <is>
+          <t>Faibles tassements diff.</t>
+        </is>
+      </c>
+      <c r="K30" s="41" t="inlineStr">
+        <is>
+          <t>EC2 / FD P18-717</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="41" t="inlineStr">
+        <is>
+          <t>FM61035X20</t>
+        </is>
+      </c>
+      <c r="B31" s="41" t="inlineStr">
+        <is>
+          <t>Semelle renforcée</t>
+        </is>
+      </c>
+      <c r="C31" s="45" t="n">
+        <v>35</v>
+      </c>
+      <c r="D31" s="45" t="n">
+        <v>20</v>
+      </c>
+      <c r="E31" s="41" t="inlineStr">
+        <is>
+          <t>6 HA 10 (2 nappes)</t>
+        </is>
+      </c>
+      <c r="F31" s="41" t="inlineStr">
+        <is>
+          <t>Cadres HA 5</t>
+        </is>
+      </c>
+      <c r="G31" s="41" t="inlineStr">
+        <is>
+          <t>e = 25</t>
+        </is>
+      </c>
+      <c r="H31" s="41" t="inlineStr">
+        <is>
+          <t>B500B</t>
+        </is>
+      </c>
+      <c r="I31" s="41" t="inlineStr">
+        <is>
+          <t>6 unités</t>
+        </is>
+      </c>
+      <c r="J31" s="43" t="inlineStr">
+        <is>
+          <t>Charges élevées</t>
+        </is>
+      </c>
+      <c r="K31" s="41" t="inlineStr">
+        <is>
+          <t>EC2 / FD P18-717</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="41" t="inlineStr">
+        <is>
+          <t>FM612140X20</t>
+        </is>
+      </c>
+      <c r="B32" s="41" t="inlineStr">
+        <is>
+          <t>Semelle renforcée</t>
+        </is>
+      </c>
+      <c r="C32" s="45" t="n">
+        <v>40</v>
+      </c>
+      <c r="D32" s="45" t="n">
+        <v>20</v>
+      </c>
+      <c r="E32" s="41" t="inlineStr">
+        <is>
+          <t>4 HA 12 + 2 HA 10</t>
+        </is>
+      </c>
+      <c r="F32" s="41" t="inlineStr">
+        <is>
+          <t>Cadres HA 5</t>
+        </is>
+      </c>
+      <c r="G32" s="41" t="inlineStr">
+        <is>
+          <t>e = 25</t>
+        </is>
+      </c>
+      <c r="H32" s="41" t="inlineStr">
+        <is>
+          <t>B500B</t>
+        </is>
+      </c>
+      <c r="I32" s="41" t="inlineStr">
+        <is>
+          <t>6 unités</t>
+        </is>
+      </c>
+      <c r="J32" s="43" t="inlineStr">
+        <is>
+          <t>Rigidité renforcée</t>
+        </is>
+      </c>
+      <c r="K32" s="41" t="inlineStr">
+        <is>
+          <t>EC2 / FD P18-717</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="39" t="inlineStr">
+        <is>
+          <t>4. CHAÎNAGES HORIZONTAUX &amp; VERTICAUX (DTU 20.1 &amp; ZONE SISMIQUE Z1 À Z4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="40" t="inlineStr">
+        <is>
+          <t>Réf. Armature</t>
+        </is>
+      </c>
+      <c r="B35" s="40" t="inlineStr">
+        <is>
+          <t>Zone Sismique</t>
+        </is>
+      </c>
+      <c r="C35" s="40" t="inlineStr">
+        <is>
+          <t>Section Béton (cm)</t>
+        </is>
+      </c>
+      <c r="D35" s="40" t="inlineStr">
+        <is>
+          <t>Aciers Filants</t>
+        </is>
+      </c>
+      <c r="E35" s="40" t="inlineStr">
+        <is>
+          <t>Section An (cm²)</t>
+        </is>
+      </c>
+      <c r="F35" s="40" t="inlineStr">
+        <is>
+          <t>Armat. Transversales</t>
+        </is>
+      </c>
+      <c r="G35" s="40" t="inlineStr">
+        <is>
+          <t>Espac. (cm)</t>
+        </is>
+      </c>
+      <c r="H35" s="40" t="inlineStr">
+        <is>
+          <t>Fermeture Cadres</t>
+        </is>
+      </c>
+      <c r="I35" s="40" t="inlineStr">
+        <is>
+          <t>Positionnement Nœud</t>
+        </is>
+      </c>
+      <c r="J35" s="40" t="inlineStr">
+        <is>
+          <t>Application</t>
+        </is>
+      </c>
+      <c r="K35" s="40" t="inlineStr">
+        <is>
+          <t>Règle Normative</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="41" t="inlineStr">
+        <is>
+          <t>CH2104X10</t>
+        </is>
+      </c>
+      <c r="B36" s="41" t="inlineStr">
+        <is>
+          <t>Z1 - Z2 (Très faible / Faible)</t>
+        </is>
+      </c>
+      <c r="C36" s="41" t="inlineStr">
+        <is>
+          <t>15 x 20</t>
+        </is>
+      </c>
+      <c r="D36" s="41" t="inlineStr">
+        <is>
+          <t>2 HA 10</t>
+        </is>
+      </c>
+      <c r="E36" s="44" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="F36" s="41" t="inlineStr">
+        <is>
+          <t>Épingles Ø 4</t>
+        </is>
+      </c>
+      <c r="G36" s="41" t="inlineStr">
+        <is>
+          <t>e = 30 à 50</t>
+        </is>
+      </c>
+      <c r="H36" s="41" t="inlineStr">
+        <is>
+          <t>Libre</t>
+        </is>
+      </c>
+      <c r="I36" s="41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J36" s="43" t="inlineStr">
+        <is>
+          <t>Chaînage horizontal / pignon</t>
+        </is>
+      </c>
+      <c r="K36" s="43" t="inlineStr">
+        <is>
+          <t>DTU 20.1 (An &gt;= 1.50 cm²)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="41" t="inlineStr">
+        <is>
+          <t>CH4710X10</t>
+        </is>
+      </c>
+      <c r="B37" s="41" t="inlineStr">
+        <is>
+          <t>Z1 - Z2 (Très faible / Faible)</t>
+        </is>
+      </c>
+      <c r="C37" s="41" t="inlineStr">
+        <is>
+          <t>15 x 15</t>
+        </is>
+      </c>
+      <c r="D37" s="41" t="inlineStr">
+        <is>
+          <t>4 HA 7</t>
+        </is>
+      </c>
+      <c r="E37" s="44" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="F37" s="41" t="inlineStr">
+        <is>
+          <t>Cadres Ø 4</t>
+        </is>
+      </c>
+      <c r="G37" s="41" t="inlineStr">
+        <is>
+          <t>e = 30 à 40</t>
+        </is>
+      </c>
+      <c r="H37" s="41" t="inlineStr">
+        <is>
+          <t>Libre</t>
+        </is>
+      </c>
+      <c r="I37" s="41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J37" s="43" t="inlineStr">
+        <is>
+          <t>Chaînage horizontal / vertical</t>
+        </is>
+      </c>
+      <c r="K37" s="43" t="inlineStr">
+        <is>
+          <t>DTU 20.1 (An &gt;= 1.50 cm²)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="41" t="inlineStr">
+        <is>
+          <t>CH4815X15</t>
+        </is>
+      </c>
+      <c r="B38" s="41" t="inlineStr">
+        <is>
+          <t>Z1 - Z2 (Très faible / Faible)</t>
+        </is>
+      </c>
+      <c r="C38" s="41" t="inlineStr">
+        <is>
+          <t>20 x 20</t>
+        </is>
+      </c>
+      <c r="D38" s="41" t="inlineStr">
+        <is>
+          <t>4 HA 8</t>
+        </is>
+      </c>
+      <c r="E38" s="44" t="n">
+        <v>2.01</v>
+      </c>
+      <c r="F38" s="41" t="inlineStr">
+        <is>
+          <t>Cadres Ø 4</t>
+        </is>
+      </c>
+      <c r="G38" s="41" t="inlineStr">
+        <is>
+          <t>e = 30 à 40</t>
+        </is>
+      </c>
+      <c r="H38" s="41" t="inlineStr">
+        <is>
+          <t>Libre</t>
+        </is>
+      </c>
+      <c r="I38" s="41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J38" s="43" t="inlineStr">
+        <is>
+          <t>Chaînage niveaux courants</t>
+        </is>
+      </c>
+      <c r="K38" s="43" t="inlineStr">
+        <is>
+          <t>DTU 20.1 (An &gt;= 1.50 cm²)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="41" t="inlineStr">
+        <is>
+          <t>CHR41010X10</t>
+        </is>
+      </c>
+      <c r="B39" s="41" t="inlineStr">
+        <is>
+          <t>Z1 - Z2 (Très faible / Faible)</t>
+        </is>
+      </c>
+      <c r="C39" s="41" t="inlineStr">
+        <is>
+          <t>20 x 20</t>
+        </is>
+      </c>
+      <c r="D39" s="41" t="inlineStr">
+        <is>
+          <t>4 HA 10</t>
+        </is>
+      </c>
+      <c r="E39" s="44" t="n">
+        <v>3.14</v>
+      </c>
+      <c r="F39" s="41" t="inlineStr">
+        <is>
+          <t>Cadres HA 5</t>
+        </is>
+      </c>
+      <c r="G39" s="41" t="inlineStr">
+        <is>
+          <t>e = 20</t>
+        </is>
+      </c>
+      <c r="H39" s="41" t="inlineStr">
+        <is>
+          <t>135° ou soudé</t>
+        </is>
+      </c>
+      <c r="I39" s="41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J39" s="43" t="inlineStr">
+        <is>
+          <t>Planchers-terrasses</t>
+        </is>
+      </c>
+      <c r="K39" s="43" t="inlineStr">
+        <is>
+          <t>DTU 20.1 (An &gt;= 3.08 cm²)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="41" t="inlineStr">
+        <is>
+          <t>CS108X8</t>
+        </is>
+      </c>
+      <c r="B40" s="41" t="inlineStr">
+        <is>
+          <t>Z3 - Z4 (Modérée / Moyenne)</t>
+        </is>
+      </c>
+      <c r="C40" s="41" t="inlineStr">
+        <is>
+          <t>15 x 15 min</t>
+        </is>
+      </c>
+      <c r="D40" s="41" t="inlineStr">
+        <is>
+          <t>4 HA 10</t>
+        </is>
+      </c>
+      <c r="E40" s="44" t="n">
+        <v>3.14</v>
+      </c>
+      <c r="F40" s="41" t="inlineStr">
+        <is>
+          <t>Cadres HA 5</t>
+        </is>
+      </c>
+      <c r="G40" s="41" t="inlineStr">
+        <is>
+          <t>e = 15</t>
+        </is>
+      </c>
+      <c r="H40" s="41" t="inlineStr">
+        <is>
+          <t>Crochets 135°</t>
+        </is>
+      </c>
+      <c r="I40" s="41" t="inlineStr">
+        <is>
+          <t>1er cadre à &lt;= 7.5 cm</t>
+        </is>
+      </c>
+      <c r="J40" s="43" t="inlineStr">
+        <is>
+          <t>Chaînage vert. / horiz. sismique</t>
+        </is>
+      </c>
+      <c r="K40" s="43" t="inlineStr">
+        <is>
+          <t>CPMI EC8 / EC8-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="41" t="inlineStr">
+        <is>
+          <t>CS1210X10</t>
+        </is>
+      </c>
+      <c r="B41" s="41" t="inlineStr">
+        <is>
+          <t>Z3 - Z4 (Modérée / Moyenne)</t>
+        </is>
+      </c>
+      <c r="C41" s="41" t="inlineStr">
+        <is>
+          <t>20 x 20 min</t>
+        </is>
+      </c>
+      <c r="D41" s="41" t="inlineStr">
+        <is>
+          <t>4 HA 12</t>
+        </is>
+      </c>
+      <c r="E41" s="44" t="n">
+        <v>4.52</v>
+      </c>
+      <c r="F41" s="41" t="inlineStr">
+        <is>
+          <t>Cadres HA 5</t>
+        </is>
+      </c>
+      <c r="G41" s="41" t="inlineStr">
+        <is>
+          <t>e = 15</t>
+        </is>
+      </c>
+      <c r="H41" s="41" t="inlineStr">
+        <is>
+          <t>Crochets 135°</t>
+        </is>
+      </c>
+      <c r="I41" s="41" t="inlineStr">
+        <is>
+          <t>1er cadre à &lt;= 7.5 cm</t>
+        </is>
+      </c>
+      <c r="J41" s="43" t="inlineStr">
+        <is>
+          <t>Chaînage vert. / horiz. sismique</t>
+        </is>
+      </c>
+      <c r="K41" s="43" t="inlineStr">
+        <is>
+          <t>CPMI EC8 / EC8-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="41" t="inlineStr">
+        <is>
+          <t>ATCS108X8</t>
+        </is>
+      </c>
+      <c r="B42" s="41" t="inlineStr">
+        <is>
+          <t>Z3 - Z4 (Modérée / Moyenne)</t>
+        </is>
+      </c>
+      <c r="C42" s="41" t="inlineStr">
+        <is>
+          <t>15 x 15 min</t>
+        </is>
+      </c>
+      <c r="D42" s="41" t="inlineStr">
+        <is>
+          <t>4 HA 10</t>
+        </is>
+      </c>
+      <c r="E42" s="44" t="n">
+        <v>3.14</v>
+      </c>
+      <c r="F42" s="41" t="inlineStr">
+        <is>
+          <t>Cadres HA 5</t>
+        </is>
+      </c>
+      <c r="G42" s="41" t="inlineStr">
+        <is>
+          <t>25-4x15-85</t>
+        </is>
+      </c>
+      <c r="H42" s="41" t="inlineStr">
+        <is>
+          <t>Crochets 135°</t>
+        </is>
+      </c>
+      <c r="I42" s="41" t="inlineStr">
+        <is>
+          <t>Recouvrement &gt;= 60 cm</t>
+        </is>
+      </c>
+      <c r="J42" s="43" t="inlineStr">
+        <is>
+          <t>Attente soubassement sismique</t>
+        </is>
+      </c>
+      <c r="K42" s="43" t="inlineStr">
+        <is>
+          <t>CPMI EC8 (HA10 &gt;= 60 cm)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="41" t="inlineStr">
+        <is>
+          <t>ATCS128X8</t>
+        </is>
+      </c>
+      <c r="B43" s="41" t="inlineStr">
+        <is>
+          <t>Z3 - Z4 (Modérée / Moyenne)</t>
+        </is>
+      </c>
+      <c r="C43" s="41" t="inlineStr">
+        <is>
+          <t>15 x 15 min</t>
+        </is>
+      </c>
+      <c r="D43" s="41" t="inlineStr">
+        <is>
+          <t>4 HA 12</t>
+        </is>
+      </c>
+      <c r="E43" s="44" t="n">
+        <v>4.52</v>
+      </c>
+      <c r="F43" s="41" t="inlineStr">
+        <is>
+          <t>Cadres HA 5</t>
+        </is>
+      </c>
+      <c r="G43" s="41" t="inlineStr">
+        <is>
+          <t>25-4x15-105</t>
+        </is>
+      </c>
+      <c r="H43" s="41" t="inlineStr">
+        <is>
+          <t>Crochets 135°</t>
+        </is>
+      </c>
+      <c r="I43" s="41" t="inlineStr">
+        <is>
+          <t>Recouvrement &gt;= 72 cm</t>
+        </is>
+      </c>
+      <c r="J43" s="43" t="inlineStr">
+        <is>
+          <t>Attente soubassement sismique</t>
+        </is>
+      </c>
+      <c r="K43" s="43" t="inlineStr">
+        <is>
+          <t>CPMI EC8 (HA12 &gt;= 72 cm)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="39" t="inlineStr">
+        <is>
+          <t>5. POUTRES À HAUTE RÉSISTANCE MANUPORTABLES (FIMUREX VULCAIN &amp; DEMETER)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="40" t="inlineStr">
+        <is>
+          <t>Réf. Poutre</t>
+        </is>
+      </c>
+      <c r="B46" s="40" t="inlineStr">
+        <is>
+          <t>Famille</t>
+        </is>
+      </c>
+      <c r="C46" s="40" t="inlineStr">
+        <is>
+          <t>Portée Franchie (cm)</t>
+        </is>
+      </c>
+      <c r="D46" s="40" t="inlineStr">
+        <is>
+          <t>Portée Réf. (cm)</t>
+        </is>
+      </c>
+      <c r="E46" s="40" t="inlineStr">
+        <is>
+          <t>Section Béton BxH</t>
+        </is>
+      </c>
+      <c r="F46" s="40" t="inlineStr">
+        <is>
+          <t>Plancher Façade (m)</t>
+        </is>
+      </c>
+      <c r="G46" s="40" t="inlineStr">
+        <is>
+          <t>Plancher Refend (m)</t>
+        </is>
+      </c>
+      <c r="H46" s="40" t="inlineStr">
+        <is>
+          <t>Pser Admissible (daN/m)</t>
+        </is>
+      </c>
+      <c r="I46" s="40" t="inlineStr">
+        <is>
+          <t>Pser Appuis (daN)</t>
+        </is>
+      </c>
+      <c r="J46" s="40" t="inlineStr">
+        <is>
+          <t>Ancrage Mini</t>
+        </is>
+      </c>
+      <c r="K46" s="40" t="inlineStr">
+        <is>
+          <t>Flèche Admissible</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="41" t="inlineStr">
+        <is>
+          <t>V25012X20</t>
+        </is>
+      </c>
+      <c r="B47" s="41" t="inlineStr">
+        <is>
+          <t>Vulcain (Refend)</t>
+        </is>
+      </c>
+      <c r="C47" s="41" t="inlineStr">
+        <is>
+          <t>160 à 210</t>
+        </is>
+      </c>
+      <c r="D47" s="45" t="n">
+        <v>200</v>
+      </c>
+      <c r="E47" s="41" t="inlineStr">
+        <is>
+          <t>20 x 25</t>
+        </is>
+      </c>
+      <c r="F47" s="44" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G47" s="44" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="H47" s="42" t="n">
+        <v>2670</v>
+      </c>
+      <c r="I47" s="42" t="n">
+        <v>2670</v>
+      </c>
+      <c r="J47" s="41" t="inlineStr">
+        <is>
+          <t>13 cm mini</t>
+        </is>
+      </c>
+      <c r="K47" s="43" t="inlineStr">
+        <is>
+          <t>L/500 (FD P18-717)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="41" t="inlineStr">
+        <is>
+          <t>V35012X25</t>
+        </is>
+      </c>
+      <c r="B48" s="41" t="inlineStr">
+        <is>
+          <t>Vulcain (Refend)</t>
+        </is>
+      </c>
+      <c r="C48" s="41" t="inlineStr">
+        <is>
+          <t>260 à 310</t>
+        </is>
+      </c>
+      <c r="D48" s="45" t="n">
+        <v>300</v>
+      </c>
+      <c r="E48" s="41" t="inlineStr">
+        <is>
+          <t>20 x 30</t>
+        </is>
+      </c>
+      <c r="F48" s="44" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="G48" s="44" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="H48" s="42" t="n">
+        <v>2650</v>
+      </c>
+      <c r="I48" s="42" t="n">
+        <v>3980</v>
+      </c>
+      <c r="J48" s="41" t="inlineStr">
+        <is>
+          <t>13 cm mini</t>
+        </is>
+      </c>
+      <c r="K48" s="43" t="inlineStr">
+        <is>
+          <t>L/500 (FD P18-717)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="41" t="inlineStr">
+        <is>
+          <t>V45012X35</t>
+        </is>
+      </c>
+      <c r="B49" s="41" t="inlineStr">
+        <is>
+          <t>Vulcain (Refend)</t>
+        </is>
+      </c>
+      <c r="C49" s="41" t="inlineStr">
+        <is>
+          <t>360 à 410</t>
+        </is>
+      </c>
+      <c r="D49" s="45" t="n">
+        <v>400</v>
+      </c>
+      <c r="E49" s="41" t="inlineStr">
+        <is>
+          <t>20 x 40</t>
+        </is>
+      </c>
+      <c r="F49" s="44" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="G49" s="44" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="H49" s="42" t="n">
+        <v>3150</v>
+      </c>
+      <c r="I49" s="42" t="n">
+        <v>6300</v>
+      </c>
+      <c r="J49" s="41" t="inlineStr">
+        <is>
+          <t>13 cm mini</t>
+        </is>
+      </c>
+      <c r="K49" s="43" t="inlineStr">
+        <is>
+          <t>L/500 (FD P18-717)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="41" t="inlineStr">
+        <is>
+          <t>V55012X40</t>
+        </is>
+      </c>
+      <c r="B50" s="41" t="inlineStr">
+        <is>
+          <t>Vulcain (Refend)</t>
+        </is>
+      </c>
+      <c r="C50" s="41" t="inlineStr">
+        <is>
+          <t>460 à 510</t>
+        </is>
+      </c>
+      <c r="D50" s="45" t="n">
+        <v>500</v>
+      </c>
+      <c r="E50" s="41" t="inlineStr">
+        <is>
+          <t>20 x 45</t>
+        </is>
+      </c>
+      <c r="F50" s="44" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="G50" s="44" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="H50" s="42" t="n">
+        <v>3040</v>
+      </c>
+      <c r="I50" s="42" t="n">
+        <v>7600</v>
+      </c>
+      <c r="J50" s="41" t="inlineStr">
+        <is>
+          <t>13 cm mini</t>
+        </is>
+      </c>
+      <c r="K50" s="43" t="inlineStr">
+        <is>
+          <t>L/500 (FD P18-717)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="41" t="inlineStr">
+        <is>
+          <t>D35014X30</t>
+        </is>
+      </c>
+      <c r="B51" s="41" t="inlineStr">
+        <is>
+          <t>Demeter (Fortes charges)</t>
+        </is>
+      </c>
+      <c r="C51" s="41" t="inlineStr">
+        <is>
+          <t>260 à 310</t>
+        </is>
+      </c>
+      <c r="D51" s="45" t="n">
+        <v>300</v>
+      </c>
+      <c r="E51" s="41" t="inlineStr">
+        <is>
+          <t>20 x 35</t>
+        </is>
+      </c>
+      <c r="F51" s="44" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="G51" s="44" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="H51" s="42" t="n">
+        <v>5190</v>
+      </c>
+      <c r="I51" s="42" t="n">
+        <v>7790</v>
+      </c>
+      <c r="J51" s="41" t="inlineStr">
+        <is>
+          <t>18 cm mini</t>
+        </is>
+      </c>
+      <c r="K51" s="43" t="inlineStr">
+        <is>
+          <t>L/500 (FD P18-717)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="41" t="inlineStr">
+        <is>
+          <t>D45014X35</t>
+        </is>
+      </c>
+      <c r="B52" s="41" t="inlineStr">
+        <is>
+          <t>Demeter (Fortes charges)</t>
+        </is>
+      </c>
+      <c r="C52" s="41" t="inlineStr">
+        <is>
+          <t>360 à 410</t>
+        </is>
+      </c>
+      <c r="D52" s="45" t="n">
+        <v>400</v>
+      </c>
+      <c r="E52" s="41" t="inlineStr">
+        <is>
+          <t>20 x 40</t>
+        </is>
+      </c>
+      <c r="F52" s="44" t="n">
+        <v>9</v>
+      </c>
+      <c r="G52" s="44" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="H52" s="42" t="n">
+        <v>4570</v>
+      </c>
+      <c r="I52" s="42" t="n">
+        <v>9140</v>
+      </c>
+      <c r="J52" s="41" t="inlineStr">
+        <is>
+          <t>18 cm mini</t>
+        </is>
+      </c>
+      <c r="K52" s="43" t="inlineStr">
+        <is>
+          <t>L/500 (FD P18-717)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="41" t="inlineStr">
+        <is>
+          <t>D55014X45</t>
+        </is>
+      </c>
+      <c r="B53" s="41" t="inlineStr">
+        <is>
+          <t>Demeter (Fortes charges)</t>
+        </is>
+      </c>
+      <c r="C53" s="41" t="inlineStr">
+        <is>
+          <t>460 à 510</t>
+        </is>
+      </c>
+      <c r="D53" s="45" t="n">
+        <v>500</v>
+      </c>
+      <c r="E53" s="41" t="inlineStr">
+        <is>
+          <t>20 x 50</t>
+        </is>
+      </c>
+      <c r="F53" s="44" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="G53" s="44" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="H53" s="42" t="n">
+        <v>4500</v>
+      </c>
+      <c r="I53" s="42" t="n">
+        <v>11250</v>
+      </c>
+      <c r="J53" s="41" t="inlineStr">
+        <is>
+          <t>18 cm mini</t>
+        </is>
+      </c>
+      <c r="K53" s="43" t="inlineStr">
+        <is>
+          <t>L/500 (FD P18-717)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="41" t="inlineStr">
+        <is>
+          <t>D65014X50</t>
+        </is>
+      </c>
+      <c r="B54" s="41" t="inlineStr">
+        <is>
+          <t>Demeter (Fortes charges)</t>
+        </is>
+      </c>
+      <c r="C54" s="41" t="inlineStr">
+        <is>
+          <t>560 à 610</t>
+        </is>
+      </c>
+      <c r="D54" s="45" t="n">
+        <v>600</v>
+      </c>
+      <c r="E54" s="41" t="inlineStr">
+        <is>
+          <t>20 x 55</t>
+        </is>
+      </c>
+      <c r="F54" s="44" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="G54" s="44" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="H54" s="42" t="n">
+        <v>3940</v>
+      </c>
+      <c r="I54" s="42" t="n">
+        <v>11820</v>
+      </c>
+      <c r="J54" s="41" t="inlineStr">
+        <is>
+          <t>18 cm mini</t>
+        </is>
+      </c>
+      <c r="K54" s="43" t="inlineStr">
+        <is>
+          <t>L/500 (FD P18-717)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="39" t="inlineStr">
+        <is>
+          <t>6. TREILLIS SOUDÉS ADETS &amp; ACCESSOIRES DE LIAISON / CONTINUITÉ</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="40" t="inlineStr">
+        <is>
+          <t>Réf. Composant</t>
+        </is>
+      </c>
+      <c r="B57" s="40" t="inlineStr">
+        <is>
+          <t>Catégorie</t>
+        </is>
+      </c>
+      <c r="C57" s="40" t="inlineStr">
+        <is>
+          <t>Dimensions / Format</t>
+        </is>
+      </c>
+      <c r="D57" s="40" t="inlineStr">
+        <is>
+          <t>Aciers / Diamètre</t>
+        </is>
+      </c>
+      <c r="E57" s="40" t="inlineStr">
+        <is>
+          <t>Maille (cm)</t>
+        </is>
+      </c>
+      <c r="F57" s="40" t="inlineStr">
+        <is>
+          <t>Poids Unitaire</t>
+        </is>
+      </c>
+      <c r="G57" s="40" t="inlineStr">
+        <is>
+          <t>Nuance Acier</t>
+        </is>
+      </c>
+      <c r="H57" s="40" t="inlineStr">
+        <is>
+          <t>Norme / Certificat</t>
+        </is>
+      </c>
+      <c r="I57" s="40" t="inlineStr">
+        <is>
+          <t>Rôle Structurel</t>
+        </is>
+      </c>
+      <c r="J57" s="40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K57" s="40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="41" t="inlineStr">
+        <is>
+          <t>ST15C</t>
+        </is>
+      </c>
+      <c r="B58" s="41" t="inlineStr">
+        <is>
+          <t>Treillis ADETS</t>
+        </is>
+      </c>
+      <c r="C58" s="41" t="inlineStr">
+        <is>
+          <t>Panneau 4.00 x 2.40 m</t>
+        </is>
+      </c>
+      <c r="D58" s="41" t="inlineStr">
+        <is>
+          <t>Filants HA 6 + HA 6</t>
+        </is>
+      </c>
+      <c r="E58" s="41" t="inlineStr">
+        <is>
+          <t>20 x 20</t>
+        </is>
+      </c>
+      <c r="F58" s="41" t="inlineStr">
+        <is>
+          <t>2.22 kg/m²</t>
+        </is>
+      </c>
+      <c r="G58" s="41" t="inlineStr">
+        <is>
+          <t>B500A / B500B</t>
+        </is>
+      </c>
+      <c r="H58" s="41" t="inlineStr">
+        <is>
+          <t>NF AFCAB / ADETS</t>
+        </is>
+      </c>
+      <c r="I58" s="43" t="inlineStr">
+        <is>
+          <t>Dallage &amp; compression</t>
+        </is>
+      </c>
+      <c r="J58" s="41" t="inlineStr"/>
+      <c r="K58" s="41" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="41" t="inlineStr">
+        <is>
+          <t>ST25C</t>
+        </is>
+      </c>
+      <c r="B59" s="41" t="inlineStr">
+        <is>
+          <t>Treillis ADETS</t>
+        </is>
+      </c>
+      <c r="C59" s="41" t="inlineStr">
+        <is>
+          <t>Panneau 6.00 x 2.40 m</t>
+        </is>
+      </c>
+      <c r="D59" s="41" t="inlineStr">
+        <is>
+          <t>Filants HA 7 + HA 7</t>
+        </is>
+      </c>
+      <c r="E59" s="41" t="inlineStr">
+        <is>
+          <t>15 x 15</t>
+        </is>
+      </c>
+      <c r="F59" s="41" t="inlineStr">
+        <is>
+          <t>4.02 kg/m²</t>
+        </is>
+      </c>
+      <c r="G59" s="41" t="inlineStr">
+        <is>
+          <t>B500B</t>
+        </is>
+      </c>
+      <c r="H59" s="41" t="inlineStr">
+        <is>
+          <t>NF AFCAB / ADETS</t>
+        </is>
+      </c>
+      <c r="I59" s="43" t="inlineStr">
+        <is>
+          <t>Structure dalle BA</t>
+        </is>
+      </c>
+      <c r="J59" s="41" t="inlineStr"/>
+      <c r="K59" s="41" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="41" t="inlineStr">
+        <is>
+          <t>ST50C</t>
+        </is>
+      </c>
+      <c r="B60" s="41" t="inlineStr">
+        <is>
+          <t>Treillis ADETS</t>
+        </is>
+      </c>
+      <c r="C60" s="41" t="inlineStr">
+        <is>
+          <t>Panneau 6.00 x 2.40 m</t>
+        </is>
+      </c>
+      <c r="D60" s="41" t="inlineStr">
+        <is>
+          <t>Filants HA 8 + HA 8</t>
+        </is>
+      </c>
+      <c r="E60" s="41" t="inlineStr">
+        <is>
+          <t>10 x 10</t>
+        </is>
+      </c>
+      <c r="F60" s="41" t="inlineStr">
+        <is>
+          <t>7.90 kg/m²</t>
+        </is>
+      </c>
+      <c r="G60" s="41" t="inlineStr">
+        <is>
+          <t>B500B</t>
+        </is>
+      </c>
+      <c r="H60" s="41" t="inlineStr">
+        <is>
+          <t>NF AFCAB / ADETS</t>
+        </is>
+      </c>
+      <c r="I60" s="43" t="inlineStr">
+        <is>
+          <t>Radiers et dalles fortes</t>
+        </is>
+      </c>
+      <c r="J60" s="41" t="inlineStr"/>
+      <c r="K60" s="41" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="41" t="inlineStr">
+        <is>
+          <t>EQ1060</t>
+        </is>
+      </c>
+      <c r="B61" s="41" t="inlineStr">
+        <is>
+          <t>Équerre de liaison</t>
+        </is>
+      </c>
+      <c r="C61" s="41" t="inlineStr">
+        <is>
+          <t>Branches 60 x 60 cm</t>
+        </is>
+      </c>
+      <c r="D61" s="41" t="inlineStr">
+        <is>
+          <t>Barre HA 10</t>
+        </is>
+      </c>
+      <c r="E61" s="41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F61" s="41" t="inlineStr">
+        <is>
+          <t>0.617 kg/ml</t>
+        </is>
+      </c>
+      <c r="G61" s="41" t="inlineStr">
+        <is>
+          <t>B500B</t>
+        </is>
+      </c>
+      <c r="H61" s="41" t="inlineStr">
+        <is>
+          <t>Eurocode 2</t>
+        </is>
+      </c>
+      <c r="I61" s="43" t="inlineStr">
+        <is>
+          <t>Liaisons d'angles chaînages</t>
+        </is>
+      </c>
+      <c r="J61" s="41" t="inlineStr"/>
+      <c r="K61" s="41" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="41" t="inlineStr">
+        <is>
+          <t>EQ1270</t>
+        </is>
+      </c>
+      <c r="B62" s="41" t="inlineStr">
+        <is>
+          <t>Équerre de liaison</t>
+        </is>
+      </c>
+      <c r="C62" s="41" t="inlineStr">
+        <is>
+          <t>Branches 70 x 70 cm</t>
+        </is>
+      </c>
+      <c r="D62" s="41" t="inlineStr">
+        <is>
+          <t>Barre HA 12</t>
+        </is>
+      </c>
+      <c r="E62" s="41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F62" s="41" t="inlineStr">
+        <is>
+          <t>0.888 kg/ml</t>
+        </is>
+      </c>
+      <c r="G62" s="41" t="inlineStr">
+        <is>
+          <t>B500B</t>
+        </is>
+      </c>
+      <c r="H62" s="41" t="inlineStr">
+        <is>
+          <t>Eurocode 2</t>
+        </is>
+      </c>
+      <c r="I62" s="43" t="inlineStr">
+        <is>
+          <t>Liaisons d'angles semelles</t>
+        </is>
+      </c>
+      <c r="J62" s="41" t="inlineStr"/>
+      <c r="K62" s="41" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="41" t="inlineStr">
+        <is>
+          <t>CD12200</t>
+        </is>
+      </c>
+      <c r="B63" s="41" t="inlineStr">
+        <is>
+          <t>Chapeau de continuité</t>
+        </is>
+      </c>
+      <c r="C63" s="41" t="inlineStr">
+        <is>
+          <t>Longueur 2.00 m</t>
+        </is>
+      </c>
+      <c r="D63" s="41" t="inlineStr">
+        <is>
+          <t>Barre HA 12</t>
+        </is>
+      </c>
+      <c r="E63" s="41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F63" s="41" t="inlineStr">
+        <is>
+          <t>0.888 kg/ml</t>
+        </is>
+      </c>
+      <c r="G63" s="41" t="inlineStr">
+        <is>
+          <t>B500B</t>
+        </is>
+      </c>
+      <c r="H63" s="41" t="inlineStr">
+        <is>
+          <t>Eurocode 2</t>
+        </is>
+      </c>
+      <c r="I63" s="43" t="inlineStr">
+        <is>
+          <t>Continuité poutrelles plancher</t>
+        </is>
+      </c>
+      <c r="J63" s="41" t="inlineStr"/>
+      <c r="K63" s="41" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="41" t="inlineStr">
+        <is>
+          <t>NOVABOX N48CX50</t>
+        </is>
+      </c>
+      <c r="B64" s="41" t="inlineStr">
+        <is>
+          <t>Boîte d'attente</t>
+        </is>
+      </c>
+      <c r="C64" s="41" t="inlineStr">
+        <is>
+          <t>Profil 0.80 m (recouv. 50 cm)</t>
+        </is>
+      </c>
+      <c r="D64" s="41" t="inlineStr">
+        <is>
+          <t>Barres HA 8 (e=200)</t>
+        </is>
+      </c>
+      <c r="E64" s="41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F64" s="41" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="G64" s="41" t="inlineStr">
+        <is>
+          <t>B500B</t>
+        </is>
+      </c>
+      <c r="H64" s="41" t="inlineStr">
+        <is>
+          <t>AFCAB R15/008</t>
+        </is>
+      </c>
+      <c r="I64" s="43" t="inlineStr">
+        <is>
+          <t>Reprise de coulage voiles/dalles</t>
+        </is>
+      </c>
+      <c r="J64" s="41" t="inlineStr"/>
+      <c r="K64" s="41" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A34:K34"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A24:K24"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A16:K16"/>
+    <mergeCell ref="A45:K45"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A56:K56"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>